<commit_message>
Update Excel data with latest changes
</commit_message>
<xml_diff>
--- a/excel_data/Hausanschluss_data.xlsx
+++ b/excel_data/Hausanschluss_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESC_LAP_RPA 2\EnergyBot_Offline\excel_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C477F45B-5BDC-4D4F-A265-57434C28601D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B980EC25-8F45-4E91-ACFD-19D2EB5E9796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3129,12 +3129,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7191,8 +7190,8 @@
       <c r="D21" t="s">
         <v>1002</v>
       </c>
-      <c r="E21" s="2">
-        <v>46082</v>
+      <c r="E21">
+        <v>1</v>
       </c>
       <c r="F21">
         <v>51.2809612</v>

</xml_diff>